<commit_message>
modified gitignore to avoid excel autosaves and added rubric template
</commit_message>
<xml_diff>
--- a/examples/ExampleRubric.xlsx
+++ b/examples/ExampleRubric.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lantagned\Box\Coursework\_Universal\DEXTER\Teams Tutorials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lantagned\Code Projects\DEXTER-Grader\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEE76C0-0127-4F1F-9AB3-1AA3D13447CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE56E5D8-74CF-43AC-98CA-79E1E80DCCBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="-16200" windowWidth="14610" windowHeight="15585" activeTab="4" xr2:uid="{15B2800C-02FD-4E9F-9C31-75FFBBECA537}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{15B2800C-02FD-4E9F-9C31-75FFBBECA537}"/>
   </bookViews>
   <sheets>
     <sheet name="Example 1" sheetId="1" r:id="rId1"/>
@@ -721,7 +721,7 @@
     <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -780,32 +780,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -867,9 +857,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -907,7 +897,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1013,7 +1003,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1155,7 +1145,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1536,7 +1526,7 @@
       </c>
       <c r="F29" s="1"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="14"/>
       <c r="B30" s="14"/>
       <c r="C30" s="10">
@@ -2221,10 +2211,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="21">
+      <c r="B2" s="25">
         <v>1</v>
       </c>
       <c r="C2" s="9">
@@ -2235,8 +2225,8 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="22"/>
-      <c r="B3" s="23"/>
+      <c r="A3" s="23"/>
+      <c r="B3" s="26"/>
       <c r="C3" s="3">
         <v>1</v>
       </c>
@@ -2245,8 +2235,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="22"/>
-      <c r="B4" s="23"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="26"/>
       <c r="C4" s="3">
         <v>1</v>
       </c>
@@ -2255,8 +2245,8 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="22"/>
-      <c r="B5" s="23"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="26"/>
       <c r="C5" s="3">
         <v>1</v>
       </c>
@@ -2265,8 +2255,8 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="23"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="26"/>
       <c r="C6" s="3">
         <v>3</v>
       </c>
@@ -2275,8 +2265,8 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
-      <c r="B7" s="23"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="3">
         <v>2</v>
       </c>
@@ -2285,8 +2275,8 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="22"/>
-      <c r="B8" s="23"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="3">
         <v>2</v>
       </c>
@@ -2295,8 +2285,8 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
-      <c r="B9" s="23"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="26"/>
       <c r="C9" s="3">
         <v>2</v>
       </c>
@@ -2305,8 +2295,8 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="22"/>
-      <c r="B10" s="23"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="26"/>
       <c r="C10" s="3">
         <v>2</v>
       </c>
@@ -2315,8 +2305,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="22"/>
-      <c r="B11" s="23"/>
+      <c r="A11" s="23"/>
+      <c r="B11" s="26"/>
       <c r="C11" s="3">
         <v>1</v>
       </c>
@@ -2325,8 +2315,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="23"/>
+      <c r="A12" s="23"/>
+      <c r="B12" s="26"/>
       <c r="C12" s="3">
         <v>2</v>
       </c>
@@ -2335,8 +2325,8 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="22"/>
-      <c r="B13" s="23"/>
+      <c r="A13" s="23"/>
+      <c r="B13" s="26"/>
       <c r="C13" s="3">
         <v>1</v>
       </c>
@@ -2346,7 +2336,7 @@
     </row>
     <row r="14" spans="1:4" s="5" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="24"/>
-      <c r="B14" s="25"/>
+      <c r="B14" s="27"/>
       <c r="C14" s="6">
         <v>1</v>
       </c>
@@ -2354,16 +2344,16 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:4" s="29" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="30"/>
-      <c r="B15" s="31"/>
-      <c r="C15" s="28"/>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="20"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="3"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="26">
         <v>1</v>
       </c>
       <c r="C16" s="10">
@@ -2374,8 +2364,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="22"/>
-      <c r="B17" s="23"/>
+      <c r="A17" s="23"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="10">
         <v>10</v>
       </c>
@@ -2384,8 +2374,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="22"/>
-      <c r="B18" s="23"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="10">
         <v>5</v>
       </c>
@@ -2598,10 +2588,10 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="27">
+      <c r="B15" s="14">
         <v>1</v>
       </c>
       <c r="C15" s="10">

</xml_diff>